<commit_message>
Back off MDP-1 wire/system claim to TBD pending neutral-bar check
After self-audit, my prior 'wire: 4 (system is 4-wire wye)' was
interpretation, not field-verified. Cover label says 277/480 V which
implies wye-with-neutral, but no one has confirmed a neutral bar in
the cabinet. Move wire to TBD so it surfaces in unknowns.md, and
rewrite the panel notes to call the interpretation out explicitly.

https://claude.ai/code/session_01QT6YAVTmLFEPkkDwgoFiBr
</commit_message>
<xml_diff>
--- a/asphalt-plant/panels/MDP-1/schedule.xlsx
+++ b/asphalt-plant/panels/MDP-1/schedule.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-04-29T04:50:04</t>
+          <t>generated 2026-05-26T04:45:24</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -641,9 +641,12 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Cover label reads "MDP-1  277/480 VOLT".
-Main breaker nameplate (Square D HCW): cat HCW1F05435-1B, 800 A, 480 V,
-3 PH, WIRE = 3 (3-pole device; panel system is 4-wire because it supplies
-277 V phase-to-neutral loads).
+Main breaker nameplate (Square D HCW): cat HCW1F05435-1B (cat # read
+from photo; not yet datasheet-confirmed), 800 A, 480 V, 3 PH, WIRE = 3
+(per nameplate). My earlier note that "WIRE = 3 means 3 conductors
+through the breaker and the system is 4-wire" was an INTERPRETATION,
+not verified. Field-verify the system wire count by opening the cabinet
+and checking for a neutral bar.
 Panel has TWO label sets: older engraved black nameplates (e.g. SOAP PUMP
 #1, TANK #3 HEAT, AC PUMP, MILL #2 AIR COMP., EPR-1) and newer orange
 labels with -P# suffixes (e.g. SOAP PUMP 1 - P7, RACK 1 PUMP - P3,

</xml_diff>

<commit_message>
Fix two unverified details found on re-review of MDP-1
- Pos 9 Soap Pump #2: the P-number I recorded as P8 was never legible
  in the photo or confirmed by the user. Backed off to TBD.
- Pos 18 Diesel Pump: the orange DIESEL PUMP - P5 label visible in the
  panel photo was omitted from the notes. Added, with the position
  pairing flagged as assumed.

https://claude.ai/code/session_01QT6YAVTmLFEPkkDwgoFiBr
</commit_message>
<xml_diff>
--- a/asphalt-plant/panels/MDP-1/schedule.xlsx
+++ b/asphalt-plant/panels/MDP-1/schedule.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-05-26T04:45:24</t>
+          <t>generated 2026-06-11T20:42:38</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>SOAP PUMP #2 (P8)</t>
+          <t>SOAP PUMP #2 (P-number TBD)</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>engraved label SOAP PUMP #2; orange label SOAP PUMP 2 - P8; close-up photo shows single-pole 20 A handle</t>
+          <t>engraved label SOAP PUMP #2; orange label SOAP PUMP 2 - P? (P-number digit not legible in photo — I previously wrote P8 without confirming it; verify in field); close-up photo shows single-pole 20 A handle. 20 A trip confirmed by user.</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>DIESEL PUMP #2 (was)</t>
+          <t>DIESEL PUMP #2 (was, P5)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>engraved label '#2 DIESEL PUMP'; removed per handwritten</t>
+          <t>engraved label '#2 DIESEL PUMP'; orange label DIESEL PUMP - P5 nearby (pairing with this position assumed, not confirmed); removed per handwritten</t>
         </is>
       </c>
     </row>

</xml_diff>